<commit_message>
Backup 2026-08: Firestore-Stand + Excel-Auswertung
</commit_message>
<xml_diff>
--- a/backup/2026-08_kataster.xlsx
+++ b/backup/2026-08_kataster.xlsx
@@ -673,8 +673,12 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="J4" t="n">
+        <v>23.5</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Katalog</t>

</xml_diff>